<commit_message>
Report: 02 March 2026
</commit_message>
<xml_diff>
--- a/reports/buy_signals_2026-03-02.xlsx
+++ b/reports/buy_signals_2026-03-02.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -630,7 +630,7 @@
         <v>1146.93</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>1147.18</v>
+        <v>1147.23</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>1814.33</v>
       </c>
       <c r="O3" s="5" t="n">
-        <v>1814.63</v>
+        <v>1814.71</v>
       </c>
     </row>
     <row r="4">
@@ -744,7 +744,7 @@
         <v>796.8200000000001</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>797.34</v>
+        <v>797.35</v>
       </c>
     </row>
     <row r="5">
@@ -801,7 +801,7 @@
         <v>425.95</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>426.04</v>
+        <v>426.06</v>
       </c>
     </row>
     <row r="6">
@@ -858,7 +858,7 @@
         <v>1259.67</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>1259.76</v>
+        <v>1259.86</v>
       </c>
     </row>
     <row r="7">
@@ -915,7 +915,7 @@
         <v>1985.58</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>1986.32</v>
+        <v>1986.46</v>
       </c>
     </row>
     <row r="8">
@@ -972,7 +972,7 @@
         <v>417.94</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>418.03</v>
+        <v>418.06</v>
       </c>
     </row>
     <row r="9">
@@ -1029,18 +1029,18 @@
         <v>469.43</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>469.45</v>
+        <v>469.46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>HONASA.NS</t>
+          <t>ATHERENERG.NS</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ATHERENERG</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2025-05-23</t>
+          <t>2025-10-21</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1059,45 +1059,45 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>288.81</v>
+        <v>678.85</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>288.88</v>
+        <v>679.45</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>288.96</v>
+        <v>680.1</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>289.03</v>
+        <v>680.4400000000001</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>289.12</v>
+        <v>680.87</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>289.21</v>
+        <v>681.08</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>289.29</v>
+        <v>681.37</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>289.38</v>
+        <v>681.58</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>289.45</v>
+        <v>681.91</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>289.46</v>
+        <v>682.16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>APOLLOHOSP.NS</t>
+          <t>HONASA.NS</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2025-10-21</t>
+          <t>2025-05-23</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1116,45 +1116,45 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>7281.35</v>
+        <v>288.81</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>7285.76</v>
+        <v>288.88</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>7289.41</v>
+        <v>288.96</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>7293.25</v>
+        <v>289.03</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>7297.9</v>
+        <v>289.12</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>7302.75</v>
+        <v>289.21</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>7308.21</v>
+        <v>289.29</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>7313.46</v>
+        <v>289.38</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>7319.1</v>
+        <v>289.45</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>7323.37</v>
+        <v>289.47</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>AMBER.NS</t>
+          <t>APOLLOHOSP.NS</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>AMBER</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2025-10-28</t>
+          <t>2025-10-21</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1173,45 +1173,45 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>6816.4</v>
+        <v>7281.35</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>6830.04</v>
+        <v>7285.76</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>6840.99</v>
+        <v>7289.41</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>6850.98</v>
+        <v>7293.25</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>6862.19</v>
+        <v>7297.9</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>6875.05</v>
+        <v>7302.75</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>6888.97</v>
+        <v>7308.21</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>6901.36</v>
+        <v>7313.46</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>6913.84</v>
+        <v>7319.1</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>6923.65</v>
+        <v>7324.29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>CENTRALBK.NS</t>
+          <t>AMBER.NS</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>CENTRALBK</t>
+          <t>AMBER</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2025-03-24</t>
+          <t>2025-10-28</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1230,45 +1230,45 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>37.16</v>
+        <v>6816.4</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>37.17</v>
+        <v>6830.04</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>37.17</v>
+        <v>6840.99</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>37.17</v>
+        <v>6850.98</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>37.18</v>
+        <v>6862.19</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>37.19</v>
+        <v>6875.05</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>37.2</v>
+        <v>6888.97</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>37.22</v>
+        <v>6901.36</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>37.23</v>
+        <v>6913.84</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>37.23</v>
+        <v>6924.99</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>SUPREMEIND.NS</t>
+          <t>CENTRALBK.NS</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>SUPREMEIND</t>
+          <t>CENTRALBK</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2025-08-22</t>
+          <t>2025-03-24</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1287,45 +1287,45 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>3830.21</v>
+        <v>37.16</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>3831.06</v>
+        <v>37.17</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>3831.4</v>
+        <v>37.17</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>3832.1</v>
+        <v>37.17</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>3832.96</v>
+        <v>37.18</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>3833.97</v>
+        <v>37.19</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>3835.68</v>
+        <v>37.2</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>3837.01</v>
+        <v>37.22</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>3838.07</v>
+        <v>37.23</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>3838.61</v>
+        <v>37.24</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>GPIL.NS</t>
+          <t>SUPREMEIND.NS</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>GPIL</t>
+          <t>SUPREMEIND</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2025-10-31</t>
+          <t>2025-08-22</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1344,45 +1344,45 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>254.58</v>
+        <v>3830.21</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>254.78</v>
+        <v>3831.06</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>254.87</v>
+        <v>3831.4</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>254.97</v>
+        <v>3832.1</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>255.15</v>
+        <v>3832.96</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>255.32</v>
+        <v>3833.97</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>255.51</v>
+        <v>3835.68</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>255.71</v>
+        <v>3837.01</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>255.84</v>
+        <v>3838.07</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>255.84</v>
+        <v>3838.96</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>TMPV.NS</t>
+          <t>GPIL.NS</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>GPIL</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2025-11-03</t>
+          <t>2025-10-31</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1401,45 +1401,45 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>364.69</v>
+        <v>254.58</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>364.94</v>
+        <v>254.78</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>365.08</v>
+        <v>254.87</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>365.25</v>
+        <v>254.97</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>365.44</v>
+        <v>255.15</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>365.59</v>
+        <v>255.32</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>365.8</v>
+        <v>255.51</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>366.12</v>
+        <v>255.71</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>366.33</v>
+        <v>255.84</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>366.33</v>
+        <v>255.84</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>INDUSINDBK.NS</t>
+          <t>TMPV.NS</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2025-03-04</t>
+          <t>2025-11-03</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1458,45 +1458,45 @@
         </is>
       </c>
       <c r="F17" s="5" t="n">
-        <v>812.97</v>
+        <v>364.69</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>813.52</v>
+        <v>364.94</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>813.99</v>
+        <v>365.08</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>814.46</v>
+        <v>365.25</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>814.89</v>
+        <v>365.44</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>815.37</v>
+        <v>365.59</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>815.87</v>
+        <v>365.8</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>816.48</v>
+        <v>366.12</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>817.05</v>
+        <v>366.33</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>817.53</v>
+        <v>366.38</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>ENGINERSIN.NS</t>
+          <t>INDUSINDBK.NS</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>ENGINERSIN</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2025-07-11</t>
+          <t>2025-03-04</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1515,45 +1515,45 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>199.38</v>
+        <v>812.97</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>199.48</v>
+        <v>813.52</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>199.6</v>
+        <v>813.99</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>199.7</v>
+        <v>814.46</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>199.81</v>
+        <v>814.89</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>199.92</v>
+        <v>815.37</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>200.04</v>
+        <v>815.87</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>200.2</v>
+        <v>816.48</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>200.33</v>
+        <v>817.05</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>200.4</v>
+        <v>817.5599999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>TRIVENI.NS</t>
+          <t>ENGINERSIN.NS</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>TRIVENI</t>
+          <t>ENGINERSIN</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>2025-05-28</t>
+          <t>2025-07-11</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1572,45 +1572,45 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>363.71</v>
+        <v>199.38</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>363.83</v>
+        <v>199.48</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>363.92</v>
+        <v>199.6</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>364.03</v>
+        <v>199.7</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>364.13</v>
+        <v>199.81</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>364.21</v>
+        <v>199.92</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>364.32</v>
+        <v>200.04</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>364.48</v>
+        <v>200.2</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>364.64</v>
+        <v>200.33</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>364.78</v>
+        <v>200.41</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>ELGIEQUIP.NS</t>
+          <t>TRIVENI.NS</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>TRIVENI</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>2025-07-24</t>
+          <t>2025-05-28</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1629,45 +1629,45 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>487.25</v>
+        <v>363.71</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>487.6</v>
+        <v>363.83</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>487.86</v>
+        <v>363.92</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>488.16</v>
+        <v>364.03</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>488.58</v>
+        <v>364.13</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>488.94</v>
+        <v>364.21</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>489.32</v>
+        <v>364.32</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>489.67</v>
+        <v>364.48</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>489.97</v>
+        <v>364.64</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>490.09</v>
+        <v>364.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>ATUL.NS</t>
+          <t>ELGIEQUIP.NS</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>2025-07-07</t>
+          <t>2025-07-24</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1686,45 +1686,45 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>6247.3</v>
+        <v>487.25</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>6249.82</v>
+        <v>487.6</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>6252.05</v>
+        <v>487.86</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>6254.13</v>
+        <v>488.16</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>6255.85</v>
+        <v>488.58</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>6257.17</v>
+        <v>488.94</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>6258.93</v>
+        <v>489.32</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>6260.59</v>
+        <v>489.67</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>6263.13</v>
+        <v>489.97</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>6264.82</v>
+        <v>490.17</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>LINDEINDIA.NS</t>
+          <t>PNB.NS</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>LINDEINDIA</t>
+          <t>PNB</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>2025-05-28</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1743,45 +1743,45 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>6332.81</v>
+        <v>123.83</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>6335.36</v>
+        <v>124.02</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>6337.83</v>
+        <v>124.11</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>6340.29</v>
+        <v>124.33</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>6342.44</v>
+        <v>124.55</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>6344.01</v>
+        <v>124.79</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>6345.96</v>
+        <v>125</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>6348.87</v>
+        <v>125.19</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>6350.88</v>
+        <v>125.33</v>
       </c>
       <c r="O22" s="5" t="n">
-        <v>6352.18</v>
+        <v>125.35</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>CCL.NS</t>
+          <t>ATUL.NS</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>CCL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>2025-11-10</t>
+          <t>2025-07-07</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -1800,45 +1800,45 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>977.75</v>
+        <v>6247.3</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>978.08</v>
+        <v>6249.82</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>978.26</v>
+        <v>6252.05</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>978.48</v>
+        <v>6254.13</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>979.22</v>
+        <v>6255.85</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>980.3200000000001</v>
+        <v>6257.17</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>981.05</v>
+        <v>6258.93</v>
       </c>
       <c r="M23" s="5" t="n">
-        <v>981.73</v>
+        <v>6260.59</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>982.16</v>
+        <v>6263.13</v>
       </c>
       <c r="O23" s="5" t="n">
-        <v>982.42</v>
+        <v>6264.76</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>NATCOPHARM.NS</t>
+          <t>LINDEINDIA.NS</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>NATCOPHARM</t>
+          <t>LINDEINDIA</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2025-05-28</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1857,45 +1857,45 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>868.66</v>
+        <v>6332.81</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>868.8099999999999</v>
+        <v>6335.36</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>868.9400000000001</v>
+        <v>6337.83</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>869.1</v>
+        <v>6340.29</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>869.26</v>
+        <v>6342.44</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>869.76</v>
+        <v>6344.01</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>870.47</v>
+        <v>6345.96</v>
       </c>
       <c r="M24" s="5" t="n">
-        <v>871.14</v>
+        <v>6348.87</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>871.9</v>
+        <v>6350.88</v>
       </c>
       <c r="O24" s="5" t="n">
-        <v>872.33</v>
+        <v>6352.52</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>SUNTV.NS</t>
+          <t>CCL.NS</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>SUNTV</t>
+          <t>CCL</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>2025-04-15</t>
+          <t>2025-11-10</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1914,45 +1914,45 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>572.55</v>
+        <v>977.75</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>572.62</v>
+        <v>978.08</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>572.65</v>
+        <v>978.26</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>572.71</v>
+        <v>978.48</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>572.77</v>
+        <v>979.22</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>572.84</v>
+        <v>980.3200000000001</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>572.99</v>
+        <v>981.05</v>
       </c>
       <c r="M25" s="5" t="n">
-        <v>573.16</v>
+        <v>981.73</v>
       </c>
       <c r="N25" s="5" t="n">
-        <v>573.5</v>
+        <v>982.16</v>
       </c>
       <c r="O25" s="5" t="n">
-        <v>573.74</v>
+        <v>982.6</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>POWERGRID.NS</t>
+          <t>NATCOPHARM.NS</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>NATCOPHARM</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>2025-04-21</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1971,45 +1971,45 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>277.71</v>
+        <v>868.66</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>277.82</v>
+        <v>868.8099999999999</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>277.9</v>
+        <v>868.9400000000001</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>278</v>
+        <v>869.1</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>278.12</v>
+        <v>869.26</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>278.24</v>
+        <v>869.76</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>278.38</v>
+        <v>870.47</v>
       </c>
       <c r="M26" s="5" t="n">
-        <v>278.49</v>
+        <v>871.14</v>
       </c>
       <c r="N26" s="5" t="n">
-        <v>278.59</v>
+        <v>871.9</v>
       </c>
       <c r="O26" s="5" t="n">
-        <v>278.65</v>
+        <v>872.4400000000001</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>AARTIIND.NS</t>
+          <t>SUNTV.NS</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>AARTIIND</t>
+          <t>SUNTV</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>2025-05-19</t>
+          <t>2025-04-15</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -2028,45 +2028,45 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>404.97</v>
+        <v>572.55</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>405.26</v>
+        <v>572.62</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>405.51</v>
+        <v>572.65</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>405.75</v>
+        <v>572.71</v>
       </c>
       <c r="J27" s="5" t="n">
-        <v>405.96</v>
+        <v>572.77</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>406.18</v>
+        <v>572.84</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>406.44</v>
+        <v>572.99</v>
       </c>
       <c r="M27" s="5" t="n">
-        <v>406.69</v>
+        <v>573.16</v>
       </c>
       <c r="N27" s="5" t="n">
-        <v>406.89</v>
+        <v>573.5</v>
       </c>
       <c r="O27" s="5" t="n">
-        <v>407.01</v>
+        <v>573.74</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>CGPOWER.NS</t>
+          <t>SYRMA.NS</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>2025-09-16</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -2085,45 +2085,45 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>686.09</v>
+        <v>769.53</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>686.3200000000001</v>
+        <v>771.03</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>686.41</v>
+        <v>772.0700000000001</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>686.65</v>
+        <v>772.96</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>686.96</v>
+        <v>773.96</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>687.3</v>
+        <v>774.72</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>687.53</v>
+        <v>775.55</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>687.88</v>
+        <v>776.35</v>
       </c>
       <c r="N28" s="5" t="n">
-        <v>688.2</v>
+        <v>776.98</v>
       </c>
       <c r="O28" s="5" t="n">
-        <v>688.3200000000001</v>
+        <v>777.04</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>ABB.NS</t>
+          <t>POWERGRID.NS</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
+          <t>2025-04-21</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -2142,45 +2142,45 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>5337.4</v>
+        <v>277.71</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>5340.49</v>
+        <v>277.82</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>5342.63</v>
+        <v>277.9</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>5346.25</v>
+        <v>278</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>5349.44</v>
+        <v>278.12</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>5353.37</v>
+        <v>278.24</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>5357.87</v>
+        <v>278.38</v>
       </c>
       <c r="M29" s="5" t="n">
-        <v>5362.12</v>
+        <v>278.49</v>
       </c>
       <c r="N29" s="5" t="n">
-        <v>5366.01</v>
+        <v>278.59</v>
       </c>
       <c r="O29" s="5" t="n">
-        <v>5368.99</v>
+        <v>278.67</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>KIMS.NS</t>
+          <t>AARTIIND.NS</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>KIMS</t>
+          <t>AARTIIND</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>2025-07-24</t>
+          <t>2025-05-19</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -2199,45 +2199,45 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>691.52</v>
+        <v>404.97</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>691.59</v>
+        <v>405.26</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>691.65</v>
+        <v>405.51</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>691.66</v>
+        <v>405.75</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>691.83</v>
+        <v>405.96</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>692.13</v>
+        <v>406.18</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>692.37</v>
+        <v>406.44</v>
       </c>
       <c r="M30" s="5" t="n">
-        <v>692.71</v>
+        <v>406.69</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>693.0599999999999</v>
+        <v>406.89</v>
       </c>
       <c r="O30" s="5" t="n">
-        <v>693.2</v>
+        <v>407.02</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>TORNTPOWER.NS</t>
+          <t>CGPOWER.NS</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>TORNTPOWER</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>2025-04-15</t>
+          <t>2025-09-16</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -2256,45 +2256,45 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>1340.49</v>
+        <v>686.09</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>1341.37</v>
+        <v>686.3200000000001</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>1342.08</v>
+        <v>686.41</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>1342.95</v>
+        <v>686.65</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>1343.84</v>
+        <v>686.96</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>1344.75</v>
+        <v>687.3</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>1345.77</v>
+        <v>687.53</v>
       </c>
       <c r="M31" s="5" t="n">
-        <v>1346.77</v>
+        <v>687.88</v>
       </c>
       <c r="N31" s="5" t="n">
-        <v>1347.77</v>
+        <v>688.2</v>
       </c>
       <c r="O31" s="5" t="n">
-        <v>1348.6</v>
+        <v>688.41</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>BANDHANBNK.NS</t>
+          <t>ABB.NS</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>BANDHANBNK</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>2025-06-30</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -2313,45 +2313,45 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>160.29</v>
+        <v>5337.4</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>160.36</v>
+        <v>5340.49</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>160.42</v>
+        <v>5342.63</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>160.49</v>
+        <v>5346.25</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>160.57</v>
+        <v>5349.44</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>160.69</v>
+        <v>5353.37</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>160.82</v>
+        <v>5357.87</v>
       </c>
       <c r="M32" s="5" t="n">
-        <v>160.97</v>
+        <v>5362.12</v>
       </c>
       <c r="N32" s="5" t="n">
-        <v>161.1</v>
+        <v>5366.01</v>
       </c>
       <c r="O32" s="5" t="n">
-        <v>161.19</v>
+        <v>5369.36</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>TIMKEN.NS</t>
+          <t>KIMS.NS</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>TIMKEN</t>
+          <t>KIMS</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-07-24</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -2370,45 +2370,45 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>3046.57</v>
+        <v>691.52</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>3047.38</v>
+        <v>691.59</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>3048.09</v>
+        <v>691.65</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>3048.83</v>
+        <v>691.66</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>3049.97</v>
+        <v>691.83</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>3051.37</v>
+        <v>692.13</v>
       </c>
       <c r="L33" s="5" t="n">
-        <v>3053.25</v>
+        <v>692.37</v>
       </c>
       <c r="M33" s="5" t="n">
-        <v>3055.3</v>
+        <v>692.71</v>
       </c>
       <c r="N33" s="5" t="n">
-        <v>3058.08</v>
+        <v>693.0599999999999</v>
       </c>
       <c r="O33" s="5" t="n">
-        <v>3059.89</v>
+        <v>693.22</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>NETWEB.NS</t>
+          <t>TORNTPOWER.NS</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>NETWEB</t>
+          <t>TORNTPOWER</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>2025-10-08</t>
+          <t>2025-04-15</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -2427,45 +2427,45 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>3372.36</v>
+        <v>1340.49</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>3372.38</v>
+        <v>1341.37</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>3374.06</v>
+        <v>1342.08</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>3376.85</v>
+        <v>1342.95</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>3378.7</v>
+        <v>1343.84</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>3380.62</v>
+        <v>1344.75</v>
       </c>
       <c r="L34" s="5" t="n">
-        <v>3383.19</v>
+        <v>1345.77</v>
       </c>
       <c r="M34" s="5" t="n">
-        <v>3386.4</v>
+        <v>1346.77</v>
       </c>
       <c r="N34" s="5" t="n">
-        <v>3391.2</v>
+        <v>1347.77</v>
       </c>
       <c r="O34" s="5" t="n">
-        <v>3394.07</v>
+        <v>1348.7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>SUNPHARMA.NS</t>
+          <t>BANDHANBNK.NS</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>BANDHANBNK</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>2025-04-28</t>
+          <t>2025-06-30</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2484,45 +2484,45 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>1679.63</v>
+        <v>160.29</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>1679.85</v>
+        <v>160.36</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>1680.02</v>
+        <v>160.42</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>1680.23</v>
+        <v>160.49</v>
       </c>
       <c r="J35" s="5" t="n">
-        <v>1680.48</v>
+        <v>160.57</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>1680.73</v>
+        <v>160.69</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>1681.12</v>
+        <v>160.82</v>
       </c>
       <c r="M35" s="5" t="n">
-        <v>1681.62</v>
+        <v>160.97</v>
       </c>
       <c r="N35" s="5" t="n">
-        <v>1681.88</v>
+        <v>161.1</v>
       </c>
       <c r="O35" s="5" t="n">
-        <v>1682.17</v>
+        <v>161.2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>ASTERDM.NS</t>
+          <t>TIMKEN.NS</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>ASTERDM</t>
+          <t>TIMKEN</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>2025-10-21</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2541,91 +2541,262 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>626.6</v>
+        <v>3046.57</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>626.63</v>
+        <v>3047.38</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>626.76</v>
+        <v>3048.09</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>626.8</v>
+        <v>3048.83</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>627.03</v>
+        <v>3049.97</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>627.15</v>
+        <v>3051.37</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>627.33</v>
+        <v>3053.25</v>
       </c>
       <c r="M36" s="5" t="n">
-        <v>627.58</v>
+        <v>3055.3</v>
       </c>
       <c r="N36" s="5" t="n">
-        <v>627.88</v>
+        <v>3058.08</v>
       </c>
       <c r="O36" s="5" t="n">
-        <v>628.01</v>
+        <v>3060.17</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
+          <t>NETWEB.NS</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>NETWEB</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-08</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>BUY / AVERAGE OUT</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>3372.36</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>3372.38</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>3374.06</v>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>3376.85</v>
+      </c>
+      <c r="J37" s="5" t="n">
+        <v>3378.7</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>3380.62</v>
+      </c>
+      <c r="L37" s="5" t="n">
+        <v>3383.19</v>
+      </c>
+      <c r="M37" s="5" t="n">
+        <v>3386.4</v>
+      </c>
+      <c r="N37" s="5" t="n">
+        <v>3391.2</v>
+      </c>
+      <c r="O37" s="5" t="n">
+        <v>3394.34</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>2025-04-28</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>BUY / AVERAGE OUT</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>1679.63</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>1679.85</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>1680.02</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>1680.23</v>
+      </c>
+      <c r="J38" s="5" t="n">
+        <v>1680.48</v>
+      </c>
+      <c r="K38" s="5" t="n">
+        <v>1680.73</v>
+      </c>
+      <c r="L38" s="5" t="n">
+        <v>1681.12</v>
+      </c>
+      <c r="M38" s="5" t="n">
+        <v>1681.62</v>
+      </c>
+      <c r="N38" s="5" t="n">
+        <v>1681.88</v>
+      </c>
+      <c r="O38" s="5" t="n">
+        <v>1682.21</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>ASTERDM.NS</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-21</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>BUY / AVERAGE OUT</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>626.6</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>626.63</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>626.76</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>626.8</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>627.03</v>
+      </c>
+      <c r="K39" s="5" t="n">
+        <v>627.15</v>
+      </c>
+      <c r="L39" s="5" t="n">
+        <v>627.33</v>
+      </c>
+      <c r="M39" s="5" t="n">
+        <v>627.58</v>
+      </c>
+      <c r="N39" s="5" t="n">
+        <v>627.88</v>
+      </c>
+      <c r="O39" s="5" t="n">
+        <v>628.0599999999999</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
           <t>HEALTHY.NS</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>HEALTHY</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>2026-01-07</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>BUY / AVERAGE OUT</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="n">
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>BUY / AVERAGE OUT</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n">
         <v>14.68</v>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="G40" s="5" t="n">
         <v>14.69</v>
       </c>
-      <c r="H37" s="5" t="n">
+      <c r="H40" s="5" t="n">
         <v>14.7</v>
       </c>
-      <c r="I37" s="5" t="n">
+      <c r="I40" s="5" t="n">
         <v>14.7</v>
       </c>
-      <c r="J37" s="5" t="n">
+      <c r="J40" s="5" t="n">
         <v>14.71</v>
       </c>
-      <c r="K37" s="5" t="n">
+      <c r="K40" s="5" t="n">
         <v>14.72</v>
       </c>
-      <c r="L37" s="5" t="n">
+      <c r="L40" s="5" t="n">
         <v>14.74</v>
       </c>
-      <c r="M37" s="5" t="n">
+      <c r="M40" s="5" t="n">
         <v>14.76</v>
       </c>
-      <c r="N37" s="5" t="n">
+      <c r="N40" s="5" t="n">
         <v>14.77</v>
       </c>
-      <c r="O37" s="5" t="n">
-        <v>14.78</v>
+      <c r="O40" s="5" t="n">
+        <v>14.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>